<commit_message>
Add table block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/table/table.css
- blocks/table/table.js
- tools/importer/import-blog-article.bundle.js
- tools/importer/import-blog-article.js
- tools/importer/parsers/table.js
- tools/importer/reports/blog/ace-pro-court-polo.report.json
- tools/importer/reports/import-blog-article.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog-article.report.xlsx
+++ b/tools/importer/reports/import-blog-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="91">
   <si>
     <t>_reportFile</t>
   </si>
@@ -175,25 +175,28 @@
     <t>blog/ace-pro-court-polo.report.json</t>
   </si>
   <si>
+    <t>["columns-feature","table"]</t>
+  </si>
+  <si>
+    <t>blog/ace-pro-court-polo</t>
+  </si>
+  <si>
+    <t>blog-article</t>
+  </si>
+  <si>
+    <t>2026-08-03T05:57:07.482Z</t>
+  </si>
+  <si>
+    <t>Court cool, street ready — the Ace Pro polo | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/ace-pro-court-polo</t>
+  </si>
+  <si>
+    <t>blog/fashion-blog-post.report.json</t>
+  </si>
+  <si>
     <t>["columns-feature"]</t>
-  </si>
-  <si>
-    <t>blog/ace-pro-court-polo</t>
-  </si>
-  <si>
-    <t>blog-article</t>
-  </si>
-  <si>
-    <t>2026-08-03T05:19:46.014Z</t>
-  </si>
-  <si>
-    <t>Court cool, street ready — the Ace Pro polo | Fashion Blog</t>
-  </si>
-  <si>
-    <t>https://wknd-trendsetters.site/blog/ace-pro-court-polo</t>
-  </si>
-  <si>
-    <t>blog/fashion-blog-post.report.json</t>
   </si>
   <si>
     <t>blog/fashion-blog-post</t>
@@ -918,10 +921,10 @@
         <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -930,24 +933,24 @@
         <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -956,24 +959,24 @@
         <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -982,24 +985,24 @@
         <v>56</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -1008,24 +1011,24 @@
         <v>56</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1034,24 +1037,24 @@
         <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1060,13 +1063,13 @@
         <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>